<commit_message>
Top-30 for tenderer: drop salt lots below 9000 RUB/t, add high-margin tube and valve lots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/TOP30_TENDERER_1210.xlsx
+++ b/TOP30_TENDERER_1210.xlsx
@@ -43,7 +43,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -141,6 +146,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1013,7 +1033,7 @@
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Объёмы смеси и соли — в документации; требования к песку и смеси</t>
+          <t>Цена за т в извещении не раскрыта: если по соли выходит меньше 9 000 ₽/т — не подаваться. Объёмы смеси и соли — в документации</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1048,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>0164300016526000497</t>
+          <t>0851300006226000106</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1038,31 +1058,31 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>44-ФЗ, аукцион</t>
+          <t>44-ФЗ, аукцион (цена за ед.)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Фабрикант</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>МБУ «Дирекция благоустройства и озеленения», Тамбов</t>
+          <t>МКУ г. Новосибирска «Дзержинка»</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Тамбовская обл.</t>
+          <t>Новосибирская обл.</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Соль для промышленных целей NaCl</t>
+          <t>Соль для промышленных целей NaCl, МКР (объём не определён, ориентир ~400 т)</t>
         </is>
       </c>
       <c r="J8" s="3" t="n">
-        <v>460</v>
+        <v>400</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
@@ -1070,19 +1090,19 @@
         </is>
       </c>
       <c r="L8" s="6" t="n">
-        <v>8500</v>
+        <v>11000</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>3910000</v>
+        <v>4400000</v>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>14.10.2026 08:00</t>
+          <t>16.10.2026 05:00</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>1%</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -1107,7 +1127,7 @@
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>Упаковка (в извещении не указана), NaCl, график поставки</t>
+          <t>Контракт с ценой за единицу; адрес — снегоотвал, ул. Профилактическая, 73</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1142,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>0851300006226000106</t>
+          <t>0318300065126000256</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1132,7 +1152,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>44-ФЗ, аукцион (цена за ед.)</t>
+          <t>44-ФЗ, аукцион</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1142,21 +1162,21 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>МКУ г. Новосибирска «Дзержинка»</t>
+          <t>МКУ Абинского ГП «Благоустройство»</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Новосибирская обл.</t>
+          <t>Краснодарский край</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Соль для промышленных целей NaCl, МКР (объём не определён, ориентир ~400 т)</t>
+          <t>Соль для промышленных целей, NaCl 96,5–97,7%, МКР ≤1 т</t>
         </is>
       </c>
       <c r="J9" s="3" t="n">
-        <v>400</v>
+        <v>150</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -1164,14 +1184,14 @@
         </is>
       </c>
       <c r="L9" s="6" t="n">
-        <v>11000</v>
+        <v>9120</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>4400000</v>
+        <v>1368000</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>16.10.2026 05:00</t>
+          <t>19.10.2026 09:00</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1201,7 +1221,7 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>Контракт с ценой за единицу; адрес — снегоотвал, ул. Профилактическая, 73</t>
+          <t>Паспорт качества: NaCl 96,5–97,7%</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1236,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>0318300065126000256</t>
+          <t>0360300052826000514</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1236,21 +1256,21 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>МКУ Абинского ГП «Благоустройство»</t>
+          <t>МБУ г. Балашов «Благоустройство и озеленение»</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Краснодарский край</t>
+          <t>Саратовская обл.</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Соль для промышленных целей, NaCl 96,5–97,7%, МКР ≤1 т</t>
+          <t>«Концентрат минеральный „Галит“»</t>
         </is>
       </c>
       <c r="J10" s="3" t="n">
-        <v>150</v>
+        <v>345</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
@@ -1258,14 +1278,14 @@
         </is>
       </c>
       <c r="L10" s="6" t="n">
-        <v>9120</v>
+        <v>10000</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>1368000</v>
+        <v>3450000</v>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>19.10.2026 09:00</t>
+          <t>13.10.2026 08:00</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -1275,7 +1295,7 @@
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1%</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
@@ -1295,7 +1315,7 @@
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>Паспорт качества: NaCl 96,5–97,7%</t>
+          <t>Допускается ли эквивалент «Галит»; срок подачи — завтра</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1330,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>9800600011626000108</t>
+          <t>0372200193426000027</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1330,21 +1350,21 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>МКУ «Бехтеевское» (Корочанский м.о.)</t>
+          <t>ГБОУ школа № 525 Московского района СПб</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Белгородская обл.</t>
+          <t>г. Санкт-Петербург</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Соль для промышленных целей NaCl</t>
+          <t>Соль для промышленных целей, мешки 20–25 кг</t>
         </is>
       </c>
       <c r="J11" s="3" t="n">
-        <v>40</v>
+        <v>6.5</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1352,24 +1372,24 @@
         </is>
       </c>
       <c r="L11" s="6" t="n">
-        <v>8800</v>
+        <v>16380</v>
       </c>
       <c r="M11" s="7" t="n">
-        <v>352000</v>
+        <v>106470</v>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>19.10.2026 08:00</t>
+          <t>16.10.2026 10:00</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
@@ -1389,7 +1409,7 @@
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>Требования к примесям сформулированы «не менее» — сверить с паспортом</t>
+          <t>Фасовка в мешки 20–25 кг</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1424,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>0360300052826000514</t>
+          <t>0142200001326018965</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1424,21 +1444,21 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>МБУ г. Балашов «Благоустройство и озеленение»</t>
+          <t>МБУ г.о. Самара «Благоустройство»</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Саратовская обл.</t>
+          <t>Самарская обл.</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>«Концентрат минеральный „Галит“»</t>
+          <t>«Концентрат минеральный „Галит“» в МКР 1 т</t>
         </is>
       </c>
       <c r="J12" s="3" t="n">
-        <v>345</v>
+        <v>11000</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1446,24 +1466,24 @@
         </is>
       </c>
       <c r="L12" s="6" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>3450000</v>
+        <v>121000000</v>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>13.10.2026 08:00</t>
+          <t>19.10.2026 11:00</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>605 000 ₽ (0,5%)</t>
         </is>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>605 000 ₽ (0,5%)</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
@@ -1473,7 +1493,7 @@
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="S12" s="3" t="inlineStr">
@@ -1483,1601 +1503,1611 @@
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>Допускается ли эквивалент «Галит»; срок подачи — завтра</t>
+          <t>Требование опыта: исполненный контракт от 24,2 млн ₽ (ПП 2571); антислеживатель</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>0118300007926000015</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>ПГР/ПГМ</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>32616449090</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>223-ФЗ, запрос котировок</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Администрация Лабинского городского поселения</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Краснодарский край</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Соль техническая, биг-бэг 1 т</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="n">
-        <v>600</v>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>ГАУК «Мосгортур»</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>г. Москва</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Противогололёдный реагент твёрдый (антиобледенитель)</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
         <is>
           <t>т</t>
         </is>
       </c>
-      <c r="L13" s="6" t="n">
-        <v>8100</v>
-      </c>
-      <c r="M13" s="7" t="n">
-        <v>4860000</v>
-      </c>
-      <c r="N13" s="3" t="inlineStr">
-        <is>
-          <t>15.10.2026</t>
-        </is>
-      </c>
-      <c r="O13" s="3" t="inlineStr">
-        <is>
-          <t>48 600 ₽ (1%)</t>
-        </is>
-      </c>
-      <c r="P13" s="3" t="inlineStr">
-        <is>
-          <t>см. извещение</t>
-        </is>
-      </c>
-      <c r="Q13" s="3" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="R13" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S13" s="3" t="inlineStr">
-        <is>
-          <t>нет (импорт допускается)</t>
-        </is>
-      </c>
-      <c r="T13" s="3" t="inlineStr">
-        <is>
-          <t>Упаковка биг-бэг 1 т; поставка до 25.12.2026</t>
+      <c r="L13" s="11" t="n">
+        <v>54490</v>
+      </c>
+      <c r="M13" s="12" t="n">
+        <v>1285964</v>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>19.10.2026 10:00</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>38 578,92 ₽ (3%)</t>
+        </is>
+      </c>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="S13" s="8" t="inlineStr">
+        <is>
+          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
+        </is>
+      </c>
+      <c r="T13" s="8" t="inlineStr">
+        <is>
+          <t>Состав, фасовка, график — в документации</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>0368300000126001453</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>ПГР/ПГМ</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>0164300016526000498</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>МБУ «Дорремстрой», Ульяновск (лот 1 из 3)</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Ульяновская обл.</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Соль техническая в МКР (~696 т)</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="n">
-        <v>696</v>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>44-ФЗ, запрос котировок</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Фабрикант</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>МБУ «Дирекция благоустройства и озеленения», Тамбов</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Тамбовская обл.</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>ПГРт многокомпонентный (≥3 веществ, ≥85%)</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>т</t>
         </is>
       </c>
-      <c r="L14" s="6" t="n">
-        <v>7180</v>
-      </c>
-      <c r="M14" s="7" t="n">
-        <v>4999000</v>
-      </c>
-      <c r="N14" s="3" t="inlineStr">
-        <is>
-          <t>15.10.2026</t>
-        </is>
-      </c>
-      <c r="O14" s="3" t="inlineStr">
-        <is>
-          <t>1%</t>
-        </is>
-      </c>
-      <c r="P14" s="3" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="Q14" s="3" t="inlineStr">
+      <c r="L14" s="11" t="n">
+        <v>61230</v>
+      </c>
+      <c r="M14" s="12" t="n">
+        <v>1836900</v>
+      </c>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>14.10.2026 08:00</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>9 184,50 ₽ (0,5%)</t>
+        </is>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="Q14" s="8" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S14" s="3" t="inlineStr">
-        <is>
-          <t>нет (импорт допускается)</t>
-        </is>
-      </c>
-      <c r="T14" s="3" t="inlineStr">
-        <is>
-          <t>Обеспечение исполнения 30% — нужна банковская гарантия</t>
+      <c r="R14" s="8" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="S14" s="8" t="inlineStr">
+        <is>
+          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
+        </is>
+      </c>
+      <c r="T14" s="8" t="inlineStr">
+        <is>
+          <t>Прочность гранул ≥3 МПа, плавящая способность ≥5 г/г, t кристаллизации ≤ −10 °C, воздействие на кожу обуви ≤10 баллов; паспорт по ГОСТ Р 58427-2020</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>0368300000126001454</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>ПГР/ПГМ</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>0164300016526000499</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>МБУ «Дорремстрой», Ульяновск (лот 2 из 3)</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Ульяновская обл.</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Соль техническая в МКР (~696 т)</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="n">
-        <v>696</v>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>МБУ «Дирекция городского хозяйства», Тамбов</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Тамбовская обл.</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>ПГРт многокомпонентный, −30 °C</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
         <is>
           <t>т</t>
         </is>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>7180</v>
-      </c>
-      <c r="M15" s="7" t="n">
-        <v>4999000</v>
-      </c>
-      <c r="N15" s="3" t="inlineStr">
-        <is>
-          <t>15.10.2026</t>
-        </is>
-      </c>
-      <c r="O15" s="3" t="inlineStr">
-        <is>
-          <t>1%</t>
-        </is>
-      </c>
-      <c r="P15" s="3" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="Q15" s="3" t="inlineStr">
+      <c r="L15" s="11" t="n">
+        <v>53840</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>732224</v>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>15.10.2026 08:00</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S15" s="3" t="inlineStr">
-        <is>
-          <t>нет (импорт допускается)</t>
-        </is>
-      </c>
-      <c r="T15" s="3" t="inlineStr">
-        <is>
-          <t>То же</t>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="R15" s="8" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="S15" s="8" t="inlineStr">
+        <is>
+          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
+        </is>
+      </c>
+      <c r="T15" s="8" t="inlineStr">
+        <is>
+          <t>Рабочая температура −30 °C; ГОСТ Р 58427-2020</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>0368300000126001455</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>ПГР/ПГМ</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>0372200258526000596</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>44-ФЗ, аукцион</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>МБУ «Дорремстрой», Ульяновск (лот 3 из 3)</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Ульяновская обл.</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Соль техническая в МКР (~696 т)</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>696</v>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>РАД</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>СПб ГБУЗ «Городская больница Св. вмч. Георгия»</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>г. Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>ПГРт с фрикционной частью (мраморная крошка), мешки 20–25 кг</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
         <is>
           <t>т</t>
         </is>
       </c>
-      <c r="L16" s="6" t="n">
-        <v>7180</v>
-      </c>
-      <c r="M16" s="7" t="n">
-        <v>4999000</v>
-      </c>
-      <c r="N16" s="3" t="inlineStr">
-        <is>
-          <t>15.10.2026</t>
-        </is>
-      </c>
-      <c r="O16" s="3" t="inlineStr">
-        <is>
-          <t>1%</t>
-        </is>
-      </c>
-      <c r="P16" s="3" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="Q16" s="3" t="inlineStr">
+      <c r="L16" s="11" t="n">
+        <v>50620</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>404960</v>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>20.10.2026</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t>см. извещение</t>
+        </is>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="Q16" s="8" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R16" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S16" s="3" t="inlineStr">
-        <is>
-          <t>нет (импорт допускается)</t>
-        </is>
-      </c>
-      <c r="T16" s="3" t="inlineStr">
-        <is>
-          <t>То же</t>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="S16" s="8" t="inlineStr">
+        <is>
+          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
+        </is>
+      </c>
+      <c r="T16" s="8" t="inlineStr">
+        <is>
+          <t>−30…−35 °C, фракция 1,5–5 мм, ГОСТ Р 58427-2020; поставки до 30.12.2027</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>0131300000626001316</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>ПГР/ПГМ</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>0373100068726000393</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>РТС-тендер</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>МБУ «Комбинат благоустройства Ленинского района», Воронеж</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Воронежская обл.</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Соль для промышленных целей NaCl ≥96,5%, помол №3, МКР (объём не определён, ориентир ~461 т)</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="n">
-        <v>461</v>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>ФГБУ «ФБ МСЭ» Минтруда России</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>г. Москва</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>ПГР твёрдый 1,5 т + щебень гранитный 2–5 мм 1 т</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
         <is>
           <t>т</t>
         </is>
       </c>
-      <c r="L17" s="6" t="n">
-        <v>7150</v>
-      </c>
-      <c r="M17" s="7" t="n">
-        <v>3296150</v>
-      </c>
-      <c r="N17" s="3" t="inlineStr">
-        <is>
-          <t>16.10.2026 09:00</t>
-        </is>
-      </c>
-      <c r="O17" s="3" t="inlineStr">
-        <is>
-          <t>32 961,50 ₽ (1%)</t>
-        </is>
-      </c>
-      <c r="P17" s="3" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="Q17" s="3" t="inlineStr">
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>105 130 / 61 770</t>
+        </is>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>219465</v>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>14.10.2026 08:00</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R17" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S17" s="3" t="inlineStr">
-        <is>
-          <t>нет (импорт допускается)</t>
-        </is>
-      </c>
-      <c r="T17" s="3" t="inlineStr">
-        <is>
-          <t>Паспорт: NaCl ≥96,5%, помол №3; адрес: ул. Острогожская, 144м</t>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="R17" s="8" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="S17" s="8" t="inlineStr">
+        <is>
+          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
+        </is>
+      </c>
+      <c r="T17" s="8" t="inlineStr">
+        <is>
+          <t>Две позиции с разной ценой</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>0128600006826000407</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Одежда / СИЗ</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>0372100027326000601</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>44-ФЗ</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>МКУ УЖКХ Александровского МО, Струнино</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Владимирская обл.</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Галит тип С, МКР 0,8–1 т</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="n">
-        <v>150</v>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="L18" s="6" t="n">
-        <v>8950</v>
-      </c>
-      <c r="M18" s="7" t="n">
-        <v>1342500</v>
-      </c>
-      <c r="N18" s="3" t="inlineStr">
-        <is>
-          <t>19.10.2026</t>
-        </is>
-      </c>
-      <c r="O18" s="3" t="inlineStr">
-        <is>
-          <t>1%</t>
-        </is>
-      </c>
-      <c r="P18" s="3" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="Q18" s="3" t="inlineStr">
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>ФБУ «Администрация …» (Санкт-Петербург)</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>г. Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>Средства индивидуальной защиты (спецодежда, термостойкие костюмы, страховочные средства)</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="n"/>
+      <c r="K18" s="13" t="inlineStr"/>
+      <c r="L18" s="13" t="inlineStr"/>
+      <c r="M18" s="16" t="n">
+        <v>18033875</v>
+      </c>
+      <c r="N18" s="13" t="inlineStr">
+        <is>
+          <t>13.10.2026 10:00</t>
+        </is>
+      </c>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>180 339 ₽ (1%)</t>
+        </is>
+      </c>
+      <c r="P18" s="13" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R18" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S18" s="3" t="inlineStr">
-        <is>
-          <t>нет (импорт допускается)</t>
-        </is>
-      </c>
-      <c r="T18" s="3" t="inlineStr">
-        <is>
-          <t>Галит тип С; поставка до 02.12.2026</t>
+      <c r="R18" s="13" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="S18" s="13" t="inlineStr">
+        <is>
+          <t>запрет на иностранные ткани/одежду/обувь — только РФ с записью ГИСП</t>
+        </is>
+      </c>
+      <c r="T18" s="13" t="inlineStr">
+        <is>
+          <t>Полный перечень позиций и характеристик — в ТЗ</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="13" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>0142300006226000073</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Одежда</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>0358200022926000030</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>44-ФЗ</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>44-ФЗ, аукцион</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>МБУ «Благоустройство», Жигулёвск</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Самарская обл.</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Соль техническая</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="n">
-        <v>145</v>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="L19" s="6" t="n">
-        <v>6870</v>
-      </c>
-      <c r="M19" s="7" t="n">
-        <v>996150</v>
-      </c>
-      <c r="N19" s="3" t="inlineStr">
-        <is>
-          <t>16.10.2026</t>
-        </is>
-      </c>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>см. извещение</t>
-        </is>
-      </c>
-      <c r="P19" s="3" t="inlineStr">
-        <is>
-          <t>см. извещение</t>
-        </is>
-      </c>
-      <c r="Q19" s="3" t="inlineStr">
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>ГКУ РО «Ростовская областная поисково-спасательная служба»</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Ростовская обл.</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>Обмундирование спасателей: летние и зимние костюмы, комбинезоны, футболки</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="n">
+        <v>1124</v>
+      </c>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>шт/компл</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>см. позиции</t>
+        </is>
+      </c>
+      <c r="M19" s="16" t="n">
+        <v>6224421</v>
+      </c>
+      <c r="N19" s="13" t="inlineStr">
+        <is>
+          <t>19.10.2026 09:00</t>
+        </is>
+      </c>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t>62 244 ₽ (1%)</t>
+        </is>
+      </c>
+      <c r="P19" s="13" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R19" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S19" s="3" t="inlineStr">
-        <is>
-          <t>нет (импорт допускается)</t>
-        </is>
-      </c>
-      <c r="T19" s="3" t="inlineStr">
-        <is>
-          <t>Упаковка и требования к NaCl</t>
+      <c r="R19" s="13" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="S19" s="13" t="inlineStr">
+        <is>
+          <t>запрет — только РФ</t>
+        </is>
+      </c>
+      <c r="T19" s="13" t="inlineStr">
+        <is>
+          <t>Цвет, шевроны, вышивка, ткани по ГОСТ</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="13" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>0372200193426000027</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Одежда</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>32616443256</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>44-ФЗ</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>223-ФЗ</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>ГБОУ школа № 525 Московского района СПб</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>г. Санкт-Петербург</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Соль для промышленных целей, мешки 20–25 кг</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="L20" s="6" t="n">
-        <v>16380</v>
-      </c>
-      <c r="M20" s="7" t="n">
-        <v>106470</v>
-      </c>
-      <c r="N20" s="3" t="inlineStr">
-        <is>
-          <t>16.10.2026 10:00</t>
-        </is>
-      </c>
-      <c r="O20" s="3" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="P20" s="3" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="Q20" s="3" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="R20" s="3" t="inlineStr">
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>ГБУ РС(Я) «ГПС РС(Я)»</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>Республика Саха (Якутия)</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>Форменная одежда: летние полевые и зимние комплекты</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="n">
+        <v>555</v>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="L20" s="17" t="n">
+        <v>9007</v>
+      </c>
+      <c r="M20" s="16" t="n">
+        <v>4999002</v>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
+        <is>
+          <t>15.10.2026 05:00</t>
+        </is>
+      </c>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="R20" s="13" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S20" s="3" t="inlineStr">
-        <is>
-          <t>нет (импорт допускается)</t>
-        </is>
-      </c>
-      <c r="T20" s="3" t="inlineStr">
-        <is>
-          <t>Фасовка в мешки 20–25 кг</t>
+      <c r="S20" s="13" t="inlineStr">
+        <is>
+          <t>запрет — только РФ</t>
+        </is>
+      </c>
+      <c r="T20" s="13" t="inlineStr">
+        <is>
+          <t>Размерная сетка, нашивки</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="13" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>0142200001326018965</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Одежда</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>32616438570</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>223-ФЗ</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>МБУ г.о. Самара «Благоустройство»</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Самарская обл.</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>«Концентрат минеральный „Галит“» в МКР 1 т</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="n">
-        <v>11000</v>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="L21" s="6" t="n">
-        <v>11000</v>
-      </c>
-      <c r="M21" s="7" t="n">
-        <v>121000000</v>
-      </c>
-      <c r="N21" s="3" t="inlineStr">
-        <is>
-          <t>19.10.2026 11:00</t>
-        </is>
-      </c>
-      <c r="O21" s="3" t="inlineStr">
-        <is>
-          <t>605 000 ₽ (0,5%)</t>
-        </is>
-      </c>
-      <c r="P21" s="3" t="inlineStr">
-        <is>
-          <t>605 000 ₽ (0,5%)</t>
-        </is>
-      </c>
-      <c r="Q21" s="3" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="R21" s="3" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="S21" s="3" t="inlineStr">
-        <is>
-          <t>нет (импорт допускается)</t>
-        </is>
-      </c>
-      <c r="T21" s="3" t="inlineStr">
-        <is>
-          <t>Требование опыта: исполненный контракт от 24,2 млн ₽ (ПП 2571); антислеживатель</t>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>ООО «Теплоэнергетическая компания – 2»</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>Московская обл.</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>Зимняя спецодежда (костюмы от пониженных температур, сварщика и др.)</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="n">
+        <v>1236</v>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>3 892 (средняя)</t>
+        </is>
+      </c>
+      <c r="M21" s="16" t="n">
+        <v>4810414</v>
+      </c>
+      <c r="N21" s="13" t="inlineStr">
+        <is>
+          <t>14.10.2026 08:00</t>
+        </is>
+      </c>
+      <c r="O21" s="13" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="P21" s="13" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="R21" s="13" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="S21" s="13" t="inlineStr">
+        <is>
+          <t>запрет — только РФ</t>
+        </is>
+      </c>
+      <c r="T21" s="13" t="inlineStr">
+        <is>
+          <t>Классы защиты по ТР ТС 019/2011</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="n">
+      <c r="A22" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>ПГР/ПГМ</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>32616449090</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>0352200022726000839</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>223-ФЗ, запрос котировок</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>ГАУК «Мосгортур»</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>г. Москва</t>
-        </is>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>Противогололёдный реагент твёрдый (антиобледенитель)</t>
-        </is>
-      </c>
-      <c r="J22" s="8" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="K22" s="8" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="L22" s="11" t="n">
-        <v>54490</v>
-      </c>
-      <c r="M22" s="12" t="n">
-        <v>1285964</v>
-      </c>
-      <c r="N22" s="8" t="inlineStr">
-        <is>
-          <t>19.10.2026 10:00</t>
-        </is>
-      </c>
-      <c r="O22" s="8" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>БУЗОО «Клинический онкологический диспансер», Омск</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Омская обл.</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови, 6 позиций (контракт на сумму, цена за ед.)</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="n"/>
+      <c r="K22" s="18" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L22" s="18" t="inlineStr">
+        <is>
+          <t>21,55–27,77</t>
+        </is>
+      </c>
+      <c r="M22" s="21" t="n">
+        <v>500000</v>
+      </c>
+      <c r="N22" s="18" t="inlineStr">
+        <is>
+          <t>15.10.2026 05:00</t>
+        </is>
+      </c>
+      <c r="O22" s="18" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
       </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>38 578,92 ₽ (3%)</t>
-        </is>
-      </c>
-      <c r="Q22" s="8" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="R22" s="8" t="inlineStr">
+      <c r="P22" s="18" t="inlineStr">
+        <is>
+          <t>10% (≈50 000 ₽)</t>
+        </is>
+      </c>
+      <c r="Q22" s="18" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="R22" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S22" s="8" t="inlineStr">
-        <is>
-          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
-        </is>
-      </c>
-      <c r="T22" s="8" t="inlineStr">
-        <is>
-          <t>Состав, фасовка, график — в документации</t>
+      <c r="S22" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T22" s="18" t="inlineStr">
+        <is>
+          <t>Крышка винтовая или двухступенчатая; контракт до 31.12.2027</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n">
+      <c r="A23" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>ПГР/ПГМ</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>0164300016526000498</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>0318300137626000326</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>44-ФЗ, запрос котировок</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
         <is>
           <t>Фабрикант</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>МБУ «Дирекция благоустройства и озеленения», Тамбов</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Тамбовская обл.</t>
-        </is>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>ПГРт многокомпонентный (≥3 веществ, ≥85%)</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="K23" s="8" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="L23" s="11" t="n">
-        <v>61230</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>1836900</v>
-      </c>
-      <c r="N23" s="8" t="inlineStr">
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Курганинская ЦРБ» МЗ КК</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="I23" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови</t>
+        </is>
+      </c>
+      <c r="J23" s="18" t="n">
+        <v>27750</v>
+      </c>
+      <c r="K23" s="18" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L23" s="22" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="M23" s="21" t="n">
+        <v>593850</v>
+      </c>
+      <c r="N23" s="18" t="inlineStr">
         <is>
           <t>14.10.2026 08:00</t>
         </is>
       </c>
-      <c r="O23" s="8" t="inlineStr">
-        <is>
-          <t>9 184,50 ₽ (0,5%)</t>
-        </is>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="Q23" s="8" t="inlineStr">
+      <c r="O23" s="18" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="P23" s="18" t="inlineStr">
+        <is>
+          <t>5% (≈29 692 ₽)</t>
+        </is>
+      </c>
+      <c r="Q23" s="18" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R23" s="8" t="inlineStr">
+      <c r="R23" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S23" s="8" t="inlineStr">
-        <is>
-          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
-        </is>
-      </c>
-      <c r="T23" s="8" t="inlineStr">
-        <is>
-          <t>Прочность гранул ≥3 МПа, плавящая способность ≥5 г/г, t кристаллизации ≤ −10 °C, воздействие на кожу обуви ≤10 баллов; паспорт по ГОСТ Р 58427-2020</t>
+      <c r="S23" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T23" s="18" t="inlineStr">
+        <is>
+          <t>Тип добавки, объём пробирки, тип крышки</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="n">
+      <c r="A24" s="18" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>ПГР/ПГМ</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>0164300016526000499</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>0318300137626000327</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>44-ФЗ</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>МБУ «Дирекция городского хозяйства», Тамбов</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>Тамбовская обл.</t>
-        </is>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>ПГРт многокомпонентный, −30 °C</t>
-        </is>
-      </c>
-      <c r="J24" s="8" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="L24" s="11" t="n">
-        <v>53840</v>
-      </c>
-      <c r="M24" s="12" t="n">
-        <v>732224</v>
-      </c>
-      <c r="N24" s="8" t="inlineStr">
-        <is>
-          <t>15.10.2026 08:00</t>
-        </is>
-      </c>
-      <c r="O24" s="8" t="inlineStr">
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>Фабрикант</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Курганинская ЦРБ» МЗ КК</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови, 2 позиции</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="n">
+        <v>27750</v>
+      </c>
+      <c r="K24" s="18" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L24" s="18" t="inlineStr">
+        <is>
+          <t>21,40 / 21,73</t>
+        </is>
+      </c>
+      <c r="M24" s="21" t="n">
+        <v>596408</v>
+      </c>
+      <c r="N24" s="18" t="inlineStr">
+        <is>
+          <t>14.10.2026 08:00</t>
+        </is>
+      </c>
+      <c r="O24" s="18" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="P24" s="18" t="inlineStr">
+        <is>
+          <t>5% (≈29 820 ₽)</t>
+        </is>
+      </c>
+      <c r="Q24" s="18" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="Q24" s="8" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="R24" s="8" t="inlineStr">
+      <c r="R24" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S24" s="8" t="inlineStr">
-        <is>
-          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
-        </is>
-      </c>
-      <c r="T24" s="8" t="inlineStr">
-        <is>
-          <t>Рабочая температура −30 °C; ГОСТ Р 58427-2020</t>
+      <c r="S24" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T24" s="18" t="inlineStr">
+        <is>
+          <t>Тип добавки и крышки; контракт до 30.12.2027</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n">
+      <c r="A25" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>ПГР/ПГМ</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>0372200258526000596</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>0318300137626000325</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>РАД</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>СПб ГБУЗ «Городская больница Св. вмч. Георгия»</t>
-        </is>
-      </c>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>г. Санкт-Петербург</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="inlineStr">
-        <is>
-          <t>ПГРт с фрикционной частью (мраморная крошка), мешки 20–25 кг</t>
-        </is>
-      </c>
-      <c r="J25" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="K25" s="8" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="L25" s="11" t="n">
-        <v>50620</v>
-      </c>
-      <c r="M25" s="12" t="n">
-        <v>404960</v>
-      </c>
-      <c r="N25" s="8" t="inlineStr">
-        <is>
-          <t>20.10.2026</t>
-        </is>
-      </c>
-      <c r="O25" s="8" t="inlineStr">
-        <is>
-          <t>см. извещение</t>
-        </is>
-      </c>
-      <c r="P25" s="8" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="Q25" s="8" t="inlineStr">
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Фабрикант</t>
+        </is>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Курганинская ЦРБ» МЗ КК</t>
+        </is>
+      </c>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="I25" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови, 3 позиции</t>
+        </is>
+      </c>
+      <c r="J25" s="18" t="n">
+        <v>28000</v>
+      </c>
+      <c r="K25" s="18" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L25" s="18" t="inlineStr">
+        <is>
+          <t>20,97–21,73</t>
+        </is>
+      </c>
+      <c r="M25" s="21" t="n">
+        <v>595655</v>
+      </c>
+      <c r="N25" s="18" t="inlineStr">
+        <is>
+          <t>14.10.2026 08:00</t>
+        </is>
+      </c>
+      <c r="O25" s="18" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="P25" s="18" t="inlineStr">
+        <is>
+          <t>5% (≈29 783 ₽)</t>
+        </is>
+      </c>
+      <c r="Q25" s="18" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R25" s="8" t="inlineStr">
+      <c r="R25" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S25" s="8" t="inlineStr">
-        <is>
-          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
-        </is>
-      </c>
-      <c r="T25" s="8" t="inlineStr">
-        <is>
-          <t>−30…−35 °C, фракция 1,5–5 мм, ГОСТ Р 58427-2020; поставки до 30.12.2027</t>
+      <c r="S25" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T25" s="18" t="inlineStr">
+        <is>
+          <t>Тип добавки и крышки; контракт до 30.12.2027</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n">
+      <c r="A26" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>ПГР/ПГМ</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>0373100068726000393</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>0318300137626000328</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="18" t="inlineStr">
         <is>
           <t>44-ФЗ</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>ФГБУ «ФБ МСЭ» Минтруда России</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>г. Москва</t>
-        </is>
-      </c>
-      <c r="I26" s="8" t="inlineStr">
-        <is>
-          <t>ПГР твёрдый 1,5 т + щебень гранитный 2–5 мм 1 т</t>
-        </is>
-      </c>
-      <c r="J26" s="8" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K26" s="8" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="L26" s="8" t="inlineStr">
-        <is>
-          <t>105 130 / 61 770</t>
-        </is>
-      </c>
-      <c r="M26" s="12" t="n">
-        <v>219465</v>
-      </c>
-      <c r="N26" s="8" t="inlineStr">
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>Фабрикант</t>
+        </is>
+      </c>
+      <c r="G26" s="18" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Курганинская ЦРБ» МЗ КК</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="I26" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови</t>
+        </is>
+      </c>
+      <c r="J26" s="18" t="n"/>
+      <c r="K26" s="18" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L26" s="18" t="inlineStr">
+        <is>
+          <t>см. извещение</t>
+        </is>
+      </c>
+      <c r="M26" s="21" t="n">
+        <v>583162</v>
+      </c>
+      <c r="N26" s="18" t="inlineStr">
         <is>
           <t>14.10.2026 08:00</t>
         </is>
       </c>
-      <c r="O26" s="8" t="inlineStr">
+      <c r="O26" s="18" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="P26" s="18" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="Q26" s="18" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="P26" s="8" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="Q26" s="8" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="R26" s="8" t="inlineStr">
+      <c r="R26" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S26" s="8" t="inlineStr">
-        <is>
-          <t>ограничение ПП 1875 — нужен российский реагент с номером реестровой записи ГИСП</t>
-        </is>
-      </c>
-      <c r="T26" s="8" t="inlineStr">
-        <is>
-          <t>Две позиции с разной ценой</t>
+      <c r="S26" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T26" s="18" t="inlineStr">
+        <is>
+          <t>Позиции, тип добавки и крышки</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n">
+      <c r="A27" s="18" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>Одежда / СИЗ</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>0372100027326000601</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>0318300100526000182</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E27" s="18" t="inlineStr">
         <is>
           <t>44-ФЗ</t>
         </is>
       </c>
-      <c r="F27" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="13" t="inlineStr">
-        <is>
-          <t>ФБУ «Администрация …» (Санкт-Петербург)</t>
-        </is>
-      </c>
-      <c r="H27" s="13" t="inlineStr">
-        <is>
-          <t>г. Санкт-Петербург</t>
-        </is>
-      </c>
-      <c r="I27" s="13" t="inlineStr">
-        <is>
-          <t>Средства индивидуальной защиты (спецодежда, термостойкие костюмы, страховочные средства)</t>
-        </is>
-      </c>
-      <c r="J27" s="13" t="n"/>
-      <c r="K27" s="13" t="inlineStr"/>
-      <c r="L27" s="13" t="inlineStr"/>
-      <c r="M27" s="16" t="n">
-        <v>18033875</v>
-      </c>
-      <c r="N27" s="13" t="inlineStr">
-        <is>
-          <t>13.10.2026 10:00</t>
-        </is>
-      </c>
-      <c r="O27" s="13" t="inlineStr">
-        <is>
-          <t>180 339 ₽ (1%)</t>
-        </is>
-      </c>
-      <c r="P27" s="13" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="Q27" s="13" t="inlineStr">
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="G27" s="18" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Тихорецкая ЦРБ» МЗ КК</t>
+        </is>
+      </c>
+      <c r="H27" s="18" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="I27" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови</t>
+        </is>
+      </c>
+      <c r="J27" s="18" t="n">
+        <v>28400</v>
+      </c>
+      <c r="K27" s="18" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L27" s="22" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="M27" s="21" t="n">
+        <v>599240</v>
+      </c>
+      <c r="N27" s="18" t="inlineStr">
+        <is>
+          <t>16.10.2026 10:00</t>
+        </is>
+      </c>
+      <c r="O27" s="18" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="P27" s="18" t="inlineStr">
+        <is>
+          <t>5% (≈29 962 ₽)</t>
+        </is>
+      </c>
+      <c r="Q27" s="18" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R27" s="13" t="inlineStr">
+      <c r="R27" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S27" s="13" t="inlineStr">
-        <is>
-          <t>запрет на иностранные ткани/одежду/обувь — только РФ с записью ГИСП</t>
-        </is>
-      </c>
-      <c r="T27" s="13" t="inlineStr">
-        <is>
-          <t>Полный перечень позиций и характеристик — в ТЗ</t>
+      <c r="S27" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T27" s="18" t="inlineStr">
+        <is>
+          <t>Тип добавки, объём, крышка</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n">
+      <c r="A28" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Одежда</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>0358200022926000030</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>0318300100526000190</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
-          <t>44-ФЗ, аукцион</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="inlineStr">
-        <is>
-          <t>ГКУ РО «Ростовская областная поисково-спасательная служба»</t>
-        </is>
-      </c>
-      <c r="H28" s="13" t="inlineStr">
-        <is>
-          <t>Ростовская обл.</t>
-        </is>
-      </c>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>Обмундирование спасателей: летние и зимние костюмы, комбинезоны, футболки</t>
-        </is>
-      </c>
-      <c r="J28" s="13" t="n">
-        <v>1124</v>
-      </c>
-      <c r="K28" s="13" t="inlineStr">
-        <is>
-          <t>шт/компл</t>
-        </is>
-      </c>
-      <c r="L28" s="13" t="inlineStr">
-        <is>
-          <t>см. позиции</t>
-        </is>
-      </c>
-      <c r="M28" s="16" t="n">
-        <v>6224421</v>
-      </c>
-      <c r="N28" s="13" t="inlineStr">
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="G28" s="18" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Тихорецкая ЦРБ» МЗ КК</t>
+        </is>
+      </c>
+      <c r="H28" s="18" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="I28" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови, 2 позиции</t>
+        </is>
+      </c>
+      <c r="J28" s="18" t="n">
+        <v>27200</v>
+      </c>
+      <c r="K28" s="18" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L28" s="18" t="inlineStr">
+        <is>
+          <t>21,10 / 22,77</t>
+        </is>
+      </c>
+      <c r="M28" s="21" t="n">
+        <v>598970</v>
+      </c>
+      <c r="N28" s="18" t="inlineStr">
         <is>
           <t>19.10.2026 09:00</t>
         </is>
       </c>
-      <c r="O28" s="13" t="inlineStr">
-        <is>
-          <t>62 244 ₽ (1%)</t>
-        </is>
-      </c>
-      <c r="P28" s="13" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="Q28" s="13" t="inlineStr">
+      <c r="O28" s="18" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="P28" s="18" t="inlineStr">
+        <is>
+          <t>5% (≈29 948 ₽)</t>
+        </is>
+      </c>
+      <c r="Q28" s="18" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R28" s="13" t="inlineStr">
+      <c r="R28" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S28" s="13" t="inlineStr">
-        <is>
-          <t>запрет — только РФ</t>
-        </is>
-      </c>
-      <c r="T28" s="13" t="inlineStr">
-        <is>
-          <t>Цвет, шевроны, вышивка, ткани по ГОСТ</t>
+      <c r="S28" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T28" s="18" t="inlineStr">
+        <is>
+          <t>Тип добавки, объём, крышка</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n">
+      <c r="A29" s="18" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>Одежда</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="inlineStr">
-        <is>
-          <t>32616443256</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>0318300100526000186</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>223-ФЗ</t>
-        </is>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="13" t="inlineStr">
-        <is>
-          <t>ГБУ РС(Я) «ГПС РС(Я)»</t>
-        </is>
-      </c>
-      <c r="H29" s="13" t="inlineStr">
-        <is>
-          <t>Республика Саха (Якутия)</t>
-        </is>
-      </c>
-      <c r="I29" s="13" t="inlineStr">
-        <is>
-          <t>Форменная одежда: летние полевые и зимние комплекты</t>
-        </is>
-      </c>
-      <c r="J29" s="13" t="n">
-        <v>555</v>
-      </c>
-      <c r="K29" s="13" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="L29" s="17" t="n">
-        <v>9007</v>
-      </c>
-      <c r="M29" s="16" t="n">
-        <v>4999002</v>
-      </c>
-      <c r="N29" s="13" t="inlineStr">
-        <is>
-          <t>15.10.2026 05:00</t>
-        </is>
-      </c>
-      <c r="O29" s="13" t="inlineStr">
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F29" s="18" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="G29" s="18" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Тихорецкая ЦРБ» МЗ КК</t>
+        </is>
+      </c>
+      <c r="H29" s="18" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="I29" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови, 2 позиции</t>
+        </is>
+      </c>
+      <c r="J29" s="18" t="n">
+        <v>24400</v>
+      </c>
+      <c r="K29" s="18" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L29" s="18" t="inlineStr">
+        <is>
+          <t>21,10 / 25,27</t>
+        </is>
+      </c>
+      <c r="M29" s="21" t="n">
+        <v>597406</v>
+      </c>
+      <c r="N29" s="18" t="inlineStr">
+        <is>
+          <t>20.10.2026 09:00</t>
+        </is>
+      </c>
+      <c r="O29" s="18" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
       </c>
-      <c r="P29" s="13" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="Q29" s="13" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="R29" s="13" t="inlineStr">
+      <c r="P29" s="18" t="inlineStr">
+        <is>
+          <t>5% (≈29 870 ₽)</t>
+        </is>
+      </c>
+      <c r="Q29" s="18" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="R29" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S29" s="13" t="inlineStr">
-        <is>
-          <t>запрет — только РФ</t>
-        </is>
-      </c>
-      <c r="T29" s="13" t="inlineStr">
-        <is>
-          <t>Размерная сетка, нашивки</t>
+      <c r="S29" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T29" s="18" t="inlineStr">
+        <is>
+          <t>Тип добавки и крышки; контракт до 16.06.2027</t>
         </is>
       </c>
     </row>
@@ -3087,12 +3117,12 @@
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Одежда</t>
+          <t>Сантехника / арматура</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>32616438570</t>
+          <t>32616442935</t>
         </is>
       </c>
       <c r="D30" s="15" t="inlineStr">
@@ -3107,26 +3137,26 @@
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ЭТП ПАО «Т Плюс»</t>
         </is>
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>ООО «Теплоэнергетическая компания – 2»</t>
+          <t>ПАО «Т Плюс», филиал «Нижегородский»</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>Московская обл.</t>
+          <t>Нижегородская обл.</t>
         </is>
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>Зимняя спецодежда (костюмы от пониженных температур, сварщика и др.)</t>
+          <t>Запорная арматура стальная для ТЭЦ (вентили ВТ-5, ВИГ, клапаны 15с27нж, 15с22нж, 19лс53нж и др.), 19 позиций</t>
         </is>
       </c>
       <c r="J30" s="13" t="n">
-        <v>1236</v>
+        <v>127</v>
       </c>
       <c r="K30" s="13" t="inlineStr">
         <is>
@@ -3135,15 +3165,15 @@
       </c>
       <c r="L30" s="13" t="inlineStr">
         <is>
-          <t>3 892 (средняя)</t>
+          <t>см. документацию</t>
         </is>
       </c>
       <c r="M30" s="16" t="n">
-        <v>4810414</v>
+        <v>1883587</v>
       </c>
       <c r="N30" s="13" t="inlineStr">
         <is>
-          <t>14.10.2026 08:00</t>
+          <t>16.10.2026 14:00</t>
         </is>
       </c>
       <c r="O30" s="13" t="inlineStr">
@@ -3163,17 +3193,17 @@
       </c>
       <c r="R30" s="13" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="S30" s="13" t="inlineStr">
         <is>
-          <t>запрет — только РФ</t>
+          <t>проверить в документации</t>
         </is>
       </c>
       <c r="T30" s="13" t="inlineStr">
         <is>
-          <t>Классы защиты по ТР ТС 019/2011</t>
+          <t>Цены по позициям в извещении нет — смотреть документацию; указана ли НМЦ без НДС; допускаются ли аналоги энергетических вентилей</t>
         </is>
       </c>
     </row>
@@ -3264,186 +3294,186 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="n">
+      <c r="A32" s="18" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B32" s="18" t="inlineStr">
         <is>
           <t>Медрасходники</t>
         </is>
       </c>
-      <c r="C32" s="14" t="inlineStr">
+      <c r="C32" s="19" t="inlineStr">
         <is>
           <t>0373200001326001396</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="E32" s="18" t="inlineStr">
         <is>
           <t>44-ФЗ, запрос котировок</t>
         </is>
       </c>
-      <c r="F32" s="13" t="inlineStr">
+      <c r="F32" s="18" t="inlineStr">
         <is>
           <t>Росэлторг</t>
         </is>
       </c>
-      <c r="G32" s="13" t="inlineStr">
+      <c r="G32" s="18" t="inlineStr">
         <is>
           <t>ГБУЗ г. Москвы «ГКБ им. В.В. Вересаева ДЗМ»</t>
         </is>
       </c>
-      <c r="H32" s="13" t="inlineStr">
+      <c r="H32" s="18" t="inlineStr">
         <is>
           <t>г. Москва</t>
         </is>
       </c>
-      <c r="I32" s="13" t="inlineStr">
+      <c r="I32" s="18" t="inlineStr">
         <is>
           <t>Пробирки вакуумные с активатором свёртывания</t>
         </is>
       </c>
-      <c r="J32" s="13" t="n">
+      <c r="J32" s="18" t="n">
         <v>150000</v>
       </c>
-      <c r="K32" s="13" t="inlineStr">
+      <c r="K32" s="18" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="L32" s="17" t="n">
+      <c r="L32" s="22" t="n">
         <v>19.68</v>
       </c>
-      <c r="M32" s="16" t="n">
+      <c r="M32" s="21" t="n">
         <v>2952000</v>
       </c>
-      <c r="N32" s="13" t="inlineStr">
+      <c r="N32" s="18" t="inlineStr">
         <is>
           <t>15.10.2026 09:00</t>
         </is>
       </c>
-      <c r="O32" s="13" t="inlineStr">
+      <c r="O32" s="18" t="inlineStr">
         <is>
           <t>14 760 ₽ (0,5%)</t>
         </is>
       </c>
-      <c r="P32" s="13" t="inlineStr">
+      <c r="P32" s="18" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="Q32" s="13" t="inlineStr">
+      <c r="Q32" s="18" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R32" s="13" t="inlineStr">
+      <c r="R32" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S32" s="13" t="inlineStr">
+      <c r="S32" s="18" t="inlineStr">
         <is>
           <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
         </is>
       </c>
-      <c r="T32" s="13" t="inlineStr">
+      <c r="T32" s="18" t="inlineStr">
         <is>
           <t>Крышка с полнозаходной резьбой или двухступенчатым снятием</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="n">
+      <c r="A33" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>Медрасходники</t>
         </is>
       </c>
-      <c r="C33" s="14" t="inlineStr">
+      <c r="C33" s="19" t="inlineStr">
         <is>
           <t>0318300254126000157</t>
         </is>
       </c>
-      <c r="D33" s="15" t="inlineStr">
+      <c r="D33" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E33" s="13" t="inlineStr">
+      <c r="E33" s="18" t="inlineStr">
         <is>
           <t>44-ФЗ</t>
         </is>
       </c>
-      <c r="F33" s="13" t="inlineStr">
+      <c r="F33" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G33" s="13" t="inlineStr">
+      <c r="G33" s="18" t="inlineStr">
         <is>
           <t>ГБУЗ (Краснодарский край)</t>
         </is>
       </c>
-      <c r="H33" s="13" t="inlineStr">
+      <c r="H33" s="18" t="inlineStr">
         <is>
           <t>Краснодарский край</t>
         </is>
       </c>
-      <c r="I33" s="13" t="inlineStr">
+      <c r="I33" s="18" t="inlineStr">
         <is>
           <t>Пробирки вакуумные / контейнеры</t>
         </is>
       </c>
-      <c r="J33" s="13" t="n"/>
-      <c r="K33" s="13" t="inlineStr">
+      <c r="J33" s="18" t="n"/>
+      <c r="K33" s="18" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="L33" s="17" t="n">
+      <c r="L33" s="22" t="n">
         <v>32.57</v>
       </c>
-      <c r="M33" s="16" t="n">
+      <c r="M33" s="21" t="n">
         <v>586260</v>
       </c>
-      <c r="N33" s="13" t="inlineStr">
+      <c r="N33" s="18" t="inlineStr">
         <is>
           <t>19.10.2026 08:00</t>
         </is>
       </c>
-      <c r="O33" s="13" t="inlineStr">
+      <c r="O33" s="18" t="inlineStr">
         <is>
           <t>см. извещение</t>
         </is>
       </c>
-      <c r="P33" s="13" t="inlineStr">
+      <c r="P33" s="18" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="Q33" s="13" t="inlineStr">
+      <c r="Q33" s="18" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="R33" s="13" t="inlineStr">
+      <c r="R33" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="S33" s="13" t="inlineStr">
+      <c r="S33" s="18" t="inlineStr">
         <is>
           <t>запрет — только РФ (реестр) + РУ</t>
         </is>
       </c>
-      <c r="T33" s="13" t="inlineStr">
+      <c r="T33" s="18" t="inlineStr">
         <is>
           <t>Объёмы, тип добавки, размер пробирки</t>
         </is>

</xml_diff>

<commit_message>
Top-30 for tenderer: drop workwear lots, add two more tube lots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/TOP30_TENDERER_1210.xlsx
+++ b/TOP30_TENDERER_1210.xlsx
@@ -1985,12 +1985,12 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Одежда / СИЗ</t>
+          <t>Форменная одежда</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>0372100027326000601</t>
+          <t>0358200022926000030</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>44-ФЗ</t>
+          <t>44-ФЗ, аукцион</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
@@ -2010,33 +2010,43 @@
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>ФБУ «Администрация …» (Санкт-Петербург)</t>
+          <t>ГКУ РО «Ростовская областная поисково-спасательная служба»</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>г. Санкт-Петербург</t>
+          <t>Ростовская обл.</t>
         </is>
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>Средства индивидуальной защиты (спецодежда, термостойкие костюмы, страховочные средства)</t>
-        </is>
-      </c>
-      <c r="J18" s="13" t="n"/>
-      <c r="K18" s="13" t="inlineStr"/>
-      <c r="L18" s="13" t="inlineStr"/>
+          <t>Обмундирование спасателей: летние и зимние костюмы, комбинезоны, футболки</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="n">
+        <v>1124</v>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>шт/компл</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>см. позиции</t>
+        </is>
+      </c>
       <c r="M18" s="16" t="n">
-        <v>18033875</v>
+        <v>6224421</v>
       </c>
       <c r="N18" s="13" t="inlineStr">
         <is>
-          <t>13.10.2026 10:00</t>
+          <t>19.10.2026 09:00</t>
         </is>
       </c>
       <c r="O18" s="13" t="inlineStr">
         <is>
-          <t>180 339 ₽ (1%)</t>
+          <t>62 244 ₽ (1%)</t>
         </is>
       </c>
       <c r="P18" s="13" t="inlineStr">
@@ -2056,12 +2066,12 @@
       </c>
       <c r="S18" s="13" t="inlineStr">
         <is>
-          <t>запрет на иностранные ткани/одежду/обувь — только РФ с записью ГИСП</t>
+          <t>запрет — только РФ</t>
         </is>
       </c>
       <c r="T18" s="13" t="inlineStr">
         <is>
-          <t>Полный перечень позиций и характеристик — в ТЗ</t>
+          <t>Цвет, шевроны, вышивка, ткани по ГОСТ</t>
         </is>
       </c>
     </row>
@@ -2071,12 +2081,12 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Одежда</t>
+          <t>Форменная одежда</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>0358200022926000030</t>
+          <t>32616443256</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
@@ -2086,7 +2096,7 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>44-ФЗ, аукцион</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
@@ -2096,53 +2106,51 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>ГКУ РО «Ростовская областная поисково-спасательная служба»</t>
+          <t>ГБУ РС(Я) «ГПС РС(Я)»</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>Ростовская обл.</t>
+          <t>Республика Саха (Якутия)</t>
         </is>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>Обмундирование спасателей: летние и зимние костюмы, комбинезоны, футболки</t>
+          <t>Форменная одежда: летние полевые и зимние комплекты</t>
         </is>
       </c>
       <c r="J19" s="13" t="n">
-        <v>1124</v>
+        <v>555</v>
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>шт/компл</t>
-        </is>
-      </c>
-      <c r="L19" s="13" t="inlineStr">
-        <is>
-          <t>см. позиции</t>
-        </is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="L19" s="17" t="n">
+        <v>9007</v>
       </c>
       <c r="M19" s="16" t="n">
-        <v>6224421</v>
+        <v>4999002</v>
       </c>
       <c r="N19" s="13" t="inlineStr">
         <is>
-          <t>19.10.2026 09:00</t>
+          <t>15.10.2026 05:00</t>
         </is>
       </c>
       <c r="O19" s="13" t="inlineStr">
         <is>
-          <t>62 244 ₽ (1%)</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="P19" s="13" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="R19" s="13" t="inlineStr">
@@ -2157,197 +2165,195 @@
       </c>
       <c r="T19" s="13" t="inlineStr">
         <is>
-          <t>Цвет, шевроны, вышивка, ткани по ГОСТ</t>
+          <t>Размерная сетка, нашивки</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="n">
+      <c r="A20" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <t>Одежда</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>32616443256</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>0352200022726000839</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>223-ФЗ</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
-        <is>
-          <t>ГБУ РС(Я) «ГПС РС(Я)»</t>
-        </is>
-      </c>
-      <c r="H20" s="13" t="inlineStr">
-        <is>
-          <t>Республика Саха (Якутия)</t>
-        </is>
-      </c>
-      <c r="I20" s="13" t="inlineStr">
-        <is>
-          <t>Форменная одежда: летние полевые и зимние комплекты</t>
-        </is>
-      </c>
-      <c r="J20" s="13" t="n">
-        <v>555</v>
-      </c>
-      <c r="K20" s="13" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="L20" s="17" t="n">
-        <v>9007</v>
-      </c>
-      <c r="M20" s="16" t="n">
-        <v>4999002</v>
-      </c>
-      <c r="N20" s="13" t="inlineStr">
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>БУЗОО «Клинический онкологический диспансер», Омск</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Омская обл.</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови, 6 позиций (контракт на сумму, цена за ед.)</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="n"/>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>21,55–27,77</t>
+        </is>
+      </c>
+      <c r="M20" s="21" t="n">
+        <v>500000</v>
+      </c>
+      <c r="N20" s="18" t="inlineStr">
         <is>
           <t>15.10.2026 05:00</t>
         </is>
       </c>
-      <c r="O20" s="13" t="inlineStr">
+      <c r="O20" s="18" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
       </c>
-      <c r="P20" s="13" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="R20" s="13" t="inlineStr">
+      <c r="P20" s="18" t="inlineStr">
+        <is>
+          <t>10% (≈50 000 ₽)</t>
+        </is>
+      </c>
+      <c r="Q20" s="18" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="R20" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S20" s="13" t="inlineStr">
-        <is>
-          <t>запрет — только РФ</t>
-        </is>
-      </c>
-      <c r="T20" s="13" t="inlineStr">
-        <is>
-          <t>Размерная сетка, нашивки</t>
+      <c r="S20" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T20" s="18" t="inlineStr">
+        <is>
+          <t>Крышка винтовая или двухступенчатая; контракт до 31.12.2027</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="n">
+      <c r="A21" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>Одежда</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>32616438570</t>
-        </is>
-      </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>0318300137626000326</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>223-ФЗ</t>
-        </is>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="13" t="inlineStr">
-        <is>
-          <t>ООО «Теплоэнергетическая компания – 2»</t>
-        </is>
-      </c>
-      <c r="H21" s="13" t="inlineStr">
-        <is>
-          <t>Московская обл.</t>
-        </is>
-      </c>
-      <c r="I21" s="13" t="inlineStr">
-        <is>
-          <t>Зимняя спецодежда (костюмы от пониженных температур, сварщика и др.)</t>
-        </is>
-      </c>
-      <c r="J21" s="13" t="n">
-        <v>1236</v>
-      </c>
-      <c r="K21" s="13" t="inlineStr">
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>Фабрикант</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Курганинская ЦРБ» МЗ КК</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="I21" s="18" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные для взятия крови</t>
+        </is>
+      </c>
+      <c r="J21" s="18" t="n">
+        <v>27750</v>
+      </c>
+      <c r="K21" s="18" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="L21" s="13" t="inlineStr">
-        <is>
-          <t>3 892 (средняя)</t>
-        </is>
-      </c>
-      <c r="M21" s="16" t="n">
-        <v>4810414</v>
-      </c>
-      <c r="N21" s="13" t="inlineStr">
+      <c r="L21" s="22" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="M21" s="21" t="n">
+        <v>593850</v>
+      </c>
+      <c r="N21" s="18" t="inlineStr">
         <is>
           <t>14.10.2026 08:00</t>
         </is>
       </c>
-      <c r="O21" s="13" t="inlineStr">
+      <c r="O21" s="18" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
       </c>
-      <c r="P21" s="13" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="R21" s="13" t="inlineStr">
+      <c r="P21" s="18" t="inlineStr">
+        <is>
+          <t>5% (≈29 692 ₽)</t>
+        </is>
+      </c>
+      <c r="Q21" s="18" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="R21" s="18" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="S21" s="13" t="inlineStr">
-        <is>
-          <t>запрет — только РФ</t>
-        </is>
-      </c>
-      <c r="T21" s="13" t="inlineStr">
-        <is>
-          <t>Классы защиты по ТР ТС 019/2011</t>
+      <c r="S21" s="18" t="inlineStr">
+        <is>
+          <t>запрет — только РФ (реестр) + РУ Росздравнадзора</t>
+        </is>
+      </c>
+      <c r="T21" s="18" t="inlineStr">
+        <is>
+          <t>Тип добавки, объём пробирки, тип крышки</t>
         </is>
       </c>
     </row>
@@ -2362,7 +2368,7 @@
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t>0352200022726000839</t>
+          <t>0318300137626000327</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
@@ -2377,25 +2383,27 @@
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>Сбербанк-АСТ</t>
+          <t>Фабрикант</t>
         </is>
       </c>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>БУЗОО «Клинический онкологический диспансер», Омск</t>
+          <t>ГБУЗ «Курганинская ЦРБ» МЗ КК</t>
         </is>
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>Омская обл.</t>
+          <t>Краснодарский край</t>
         </is>
       </c>
       <c r="I22" s="18" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные для взятия крови, 6 позиций (контракт на сумму, цена за ед.)</t>
-        </is>
-      </c>
-      <c r="J22" s="18" t="n"/>
+          <t>Пробирки вакуумные для взятия крови, 2 позиции</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="n">
+        <v>27750</v>
+      </c>
       <c r="K22" s="18" t="inlineStr">
         <is>
           <t>шт</t>
@@ -2403,15 +2411,15 @@
       </c>
       <c r="L22" s="18" t="inlineStr">
         <is>
-          <t>21,55–27,77</t>
+          <t>21,40 / 21,73</t>
         </is>
       </c>
       <c r="M22" s="21" t="n">
-        <v>500000</v>
+        <v>596408</v>
       </c>
       <c r="N22" s="18" t="inlineStr">
         <is>
-          <t>15.10.2026 05:00</t>
+          <t>14.10.2026 08:00</t>
         </is>
       </c>
       <c r="O22" s="18" t="inlineStr">
@@ -2421,7 +2429,7 @@
       </c>
       <c r="P22" s="18" t="inlineStr">
         <is>
-          <t>10% (≈50 000 ₽)</t>
+          <t>5% (≈29 820 ₽)</t>
         </is>
       </c>
       <c r="Q22" s="18" t="inlineStr">
@@ -2441,7 +2449,7 @@
       </c>
       <c r="T22" s="18" t="inlineStr">
         <is>
-          <t>Крышка винтовая или двухступенчатая; контракт до 31.12.2027</t>
+          <t>Тип добавки и крышки; контракт до 30.12.2027</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2464,7 @@
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>0318300137626000326</t>
+          <t>0318300137626000325</t>
         </is>
       </c>
       <c r="D23" s="20" t="inlineStr">
@@ -2486,22 +2494,24 @@
       </c>
       <c r="I23" s="18" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные для взятия крови</t>
+          <t>Пробирки вакуумные для взятия крови, 3 позиции</t>
         </is>
       </c>
       <c r="J23" s="18" t="n">
-        <v>27750</v>
+        <v>28000</v>
       </c>
       <c r="K23" s="18" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="L23" s="22" t="n">
-        <v>21.4</v>
+      <c r="L23" s="18" t="inlineStr">
+        <is>
+          <t>20,97–21,73</t>
+        </is>
       </c>
       <c r="M23" s="21" t="n">
-        <v>593850</v>
+        <v>595655</v>
       </c>
       <c r="N23" s="18" t="inlineStr">
         <is>
@@ -2515,7 +2525,7 @@
       </c>
       <c r="P23" s="18" t="inlineStr">
         <is>
-          <t>5% (≈29 692 ₽)</t>
+          <t>5% (≈29 783 ₽)</t>
         </is>
       </c>
       <c r="Q23" s="18" t="inlineStr">
@@ -2535,7 +2545,7 @@
       </c>
       <c r="T23" s="18" t="inlineStr">
         <is>
-          <t>Тип добавки, объём пробирки, тип крышки</t>
+          <t>Тип добавки и крышки; контракт до 30.12.2027</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2560,7 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>0318300137626000327</t>
+          <t>0318300137626000328</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -2580,12 +2590,10 @@
       </c>
       <c r="I24" s="18" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные для взятия крови, 2 позиции</t>
-        </is>
-      </c>
-      <c r="J24" s="18" t="n">
-        <v>27750</v>
-      </c>
+          <t>Пробирки вакуумные для взятия крови</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="n"/>
       <c r="K24" s="18" t="inlineStr">
         <is>
           <t>шт</t>
@@ -2593,11 +2601,11 @@
       </c>
       <c r="L24" s="18" t="inlineStr">
         <is>
-          <t>21,40 / 21,73</t>
+          <t>см. извещение</t>
         </is>
       </c>
       <c r="M24" s="21" t="n">
-        <v>596408</v>
+        <v>583162</v>
       </c>
       <c r="N24" s="18" t="inlineStr">
         <is>
@@ -2611,7 +2619,7 @@
       </c>
       <c r="P24" s="18" t="inlineStr">
         <is>
-          <t>5% (≈29 820 ₽)</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="Q24" s="18" t="inlineStr">
@@ -2631,7 +2639,7 @@
       </c>
       <c r="T24" s="18" t="inlineStr">
         <is>
-          <t>Тип добавки и крышки; контракт до 30.12.2027</t>
+          <t>Позиции, тип добавки и крышки</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2654,7 @@
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>0318300137626000325</t>
+          <t>0318300100526000182</t>
         </is>
       </c>
       <c r="D25" s="20" t="inlineStr">
@@ -2661,12 +2669,12 @@
       </c>
       <c r="F25" s="18" t="inlineStr">
         <is>
-          <t>Фабрикант</t>
+          <t>РТС-тендер</t>
         </is>
       </c>
       <c r="G25" s="18" t="inlineStr">
         <is>
-          <t>ГБУЗ «Курганинская ЦРБ» МЗ КК</t>
+          <t>ГБУЗ «Тихорецкая ЦРБ» МЗ КК</t>
         </is>
       </c>
       <c r="H25" s="18" t="inlineStr">
@@ -2676,28 +2684,26 @@
       </c>
       <c r="I25" s="18" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные для взятия крови, 3 позиции</t>
+          <t>Пробирки вакуумные для взятия крови</t>
         </is>
       </c>
       <c r="J25" s="18" t="n">
-        <v>28000</v>
+        <v>28400</v>
       </c>
       <c r="K25" s="18" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="L25" s="18" t="inlineStr">
-        <is>
-          <t>20,97–21,73</t>
-        </is>
+      <c r="L25" s="22" t="n">
+        <v>21.1</v>
       </c>
       <c r="M25" s="21" t="n">
-        <v>595655</v>
+        <v>599240</v>
       </c>
       <c r="N25" s="18" t="inlineStr">
         <is>
-          <t>14.10.2026 08:00</t>
+          <t>16.10.2026 10:00</t>
         </is>
       </c>
       <c r="O25" s="18" t="inlineStr">
@@ -2707,7 +2713,7 @@
       </c>
       <c r="P25" s="18" t="inlineStr">
         <is>
-          <t>5% (≈29 783 ₽)</t>
+          <t>5% (≈29 962 ₽)</t>
         </is>
       </c>
       <c r="Q25" s="18" t="inlineStr">
@@ -2727,7 +2733,7 @@
       </c>
       <c r="T25" s="18" t="inlineStr">
         <is>
-          <t>Тип добавки и крышки; контракт до 30.12.2027</t>
+          <t>Тип добавки, объём, крышка</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2748,7 @@
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>0318300137626000328</t>
+          <t>0318300100526000190</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
@@ -2757,12 +2763,12 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>Фабрикант</t>
+          <t>РТС-тендер</t>
         </is>
       </c>
       <c r="G26" s="18" t="inlineStr">
         <is>
-          <t>ГБУЗ «Курганинская ЦРБ» МЗ КК</t>
+          <t>ГБУЗ «Тихорецкая ЦРБ» МЗ КК</t>
         </is>
       </c>
       <c r="H26" s="18" t="inlineStr">
@@ -2772,10 +2778,12 @@
       </c>
       <c r="I26" s="18" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные для взятия крови</t>
-        </is>
-      </c>
-      <c r="J26" s="18" t="n"/>
+          <t>Пробирки вакуумные для взятия крови, 2 позиции</t>
+        </is>
+      </c>
+      <c r="J26" s="18" t="n">
+        <v>27200</v>
+      </c>
       <c r="K26" s="18" t="inlineStr">
         <is>
           <t>шт</t>
@@ -2783,15 +2791,15 @@
       </c>
       <c r="L26" s="18" t="inlineStr">
         <is>
-          <t>см. извещение</t>
+          <t>21,10 / 22,77</t>
         </is>
       </c>
       <c r="M26" s="21" t="n">
-        <v>583162</v>
+        <v>598970</v>
       </c>
       <c r="N26" s="18" t="inlineStr">
         <is>
-          <t>14.10.2026 08:00</t>
+          <t>19.10.2026 09:00</t>
         </is>
       </c>
       <c r="O26" s="18" t="inlineStr">
@@ -2801,7 +2809,7 @@
       </c>
       <c r="P26" s="18" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>5% (≈29 948 ₽)</t>
         </is>
       </c>
       <c r="Q26" s="18" t="inlineStr">
@@ -2821,7 +2829,7 @@
       </c>
       <c r="T26" s="18" t="inlineStr">
         <is>
-          <t>Позиции, тип добавки и крышки</t>
+          <t>Тип добавки, объём, крышка</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2844,7 @@
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>0318300100526000182</t>
+          <t>0318300100526000186</t>
         </is>
       </c>
       <c r="D27" s="20" t="inlineStr">
@@ -2866,26 +2874,28 @@
       </c>
       <c r="I27" s="18" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные для взятия крови</t>
+          <t>Пробирки вакуумные для взятия крови, 2 позиции</t>
         </is>
       </c>
       <c r="J27" s="18" t="n">
-        <v>28400</v>
+        <v>24400</v>
       </c>
       <c r="K27" s="18" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="L27" s="22" t="n">
-        <v>21.1</v>
+      <c r="L27" s="18" t="inlineStr">
+        <is>
+          <t>21,10 / 25,27</t>
+        </is>
       </c>
       <c r="M27" s="21" t="n">
-        <v>599240</v>
+        <v>597406</v>
       </c>
       <c r="N27" s="18" t="inlineStr">
         <is>
-          <t>16.10.2026 10:00</t>
+          <t>20.10.2026 09:00</t>
         </is>
       </c>
       <c r="O27" s="18" t="inlineStr">
@@ -2895,7 +2905,7 @@
       </c>
       <c r="P27" s="18" t="inlineStr">
         <is>
-          <t>5% (≈29 962 ₽)</t>
+          <t>5% (≈29 870 ₽)</t>
         </is>
       </c>
       <c r="Q27" s="18" t="inlineStr">
@@ -2915,7 +2925,7 @@
       </c>
       <c r="T27" s="18" t="inlineStr">
         <is>
-          <t>Тип добавки, объём, крышка</t>
+          <t>Тип добавки и крышки; контракт до 16.06.2027</t>
         </is>
       </c>
     </row>
@@ -2930,7 +2940,7 @@
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>0318300100526000190</t>
+          <t>0318300137626000329</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
@@ -2945,12 +2955,12 @@
       </c>
       <c r="F28" s="18" t="inlineStr">
         <is>
-          <t>РТС-тендер</t>
+          <t>Фабрикант</t>
         </is>
       </c>
       <c r="G28" s="18" t="inlineStr">
         <is>
-          <t>ГБУЗ «Тихорецкая ЦРБ» МЗ КК</t>
+          <t>ГБУЗ «Курганинская ЦРБ» МЗ КК</t>
         </is>
       </c>
       <c r="H28" s="18" t="inlineStr">
@@ -2960,28 +2970,26 @@
       </c>
       <c r="I28" s="18" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные для взятия крови, 2 позиции</t>
+          <t>Пробирки вакуумные для взятия крови</t>
         </is>
       </c>
       <c r="J28" s="18" t="n">
-        <v>27200</v>
+        <v>26000</v>
       </c>
       <c r="K28" s="18" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="L28" s="18" t="inlineStr">
-        <is>
-          <t>21,10 / 22,77</t>
-        </is>
+      <c r="L28" s="22" t="n">
+        <v>21.73</v>
       </c>
       <c r="M28" s="21" t="n">
-        <v>598970</v>
+        <v>564980</v>
       </c>
       <c r="N28" s="18" t="inlineStr">
         <is>
-          <t>19.10.2026 09:00</t>
+          <t>14.10.2026 08:00</t>
         </is>
       </c>
       <c r="O28" s="18" t="inlineStr">
@@ -2991,7 +2999,7 @@
       </c>
       <c r="P28" s="18" t="inlineStr">
         <is>
-          <t>5% (≈29 948 ₽)</t>
+          <t>5% (≈28 249 ₽)</t>
         </is>
       </c>
       <c r="Q28" s="18" t="inlineStr">
@@ -3011,7 +3019,7 @@
       </c>
       <c r="T28" s="18" t="inlineStr">
         <is>
-          <t>Тип добавки, объём, крышка</t>
+          <t>Тип добавки и крышки; контракт до 30.12.2027</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3034,7 @@
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>0318300100526000186</t>
+          <t>0318300100526000191</t>
         </is>
       </c>
       <c r="D29" s="20" t="inlineStr">
@@ -3056,28 +3064,26 @@
       </c>
       <c r="I29" s="18" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные для взятия крови, 2 позиции</t>
+          <t>Пробирки вакуумные для взятия крови</t>
         </is>
       </c>
       <c r="J29" s="18" t="n">
-        <v>24400</v>
+        <v>23700</v>
       </c>
       <c r="K29" s="18" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="L29" s="18" t="inlineStr">
-        <is>
-          <t>21,10 / 25,27</t>
-        </is>
+      <c r="L29" s="22" t="n">
+        <v>25.27</v>
       </c>
       <c r="M29" s="21" t="n">
-        <v>597406</v>
+        <v>598899</v>
       </c>
       <c r="N29" s="18" t="inlineStr">
         <is>
-          <t>20.10.2026 09:00</t>
+          <t>21.10.2026 09:00</t>
         </is>
       </c>
       <c r="O29" s="18" t="inlineStr">
@@ -3087,7 +3093,7 @@
       </c>
       <c r="P29" s="18" t="inlineStr">
         <is>
-          <t>5% (≈29 870 ₽)</t>
+          <t>5% (≈29 945 ₽)</t>
         </is>
       </c>
       <c r="Q29" s="18" t="inlineStr">
@@ -3107,7 +3113,7 @@
       </c>
       <c r="T29" s="18" t="inlineStr">
         <is>
-          <t>Тип добавки и крышки; контракт до 16.06.2027</t>
+          <t>Тип добавки, объём, крышка</t>
         </is>
       </c>
     </row>

</xml_diff>